<commit_message>
Eligiendo el modelo optimo en funcion del smape
</commit_message>
<xml_diff>
--- a/Estimacion_error/datos_aves_marinas/2025/abril/RLOF/conteos_reales.xlsx
+++ b/Estimacion_error/datos_aves_marinas/2025/abril/RLOF/conteos_reales.xlsx
@@ -1,31 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renzo\Desktop\Data_Saiensss\Estadística\Trabajos (laborales)\BMAP\Proyectos\conteo-aves-bmap\Estimacion_error\datos_aves_marinas\2025\abril\RLOF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renzo\Desktop\Estadística\Trabajos (laborales)\BMAP\Proyectos\conteo-aves-bmap\Estimacion_error\datos_aves_marinas\2025\abril\RLOF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF212861-595F-47C0-B57F-54881F91DC8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB89041-2E0D-4E98-B98E-A968A2768042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
+    <sheet name="Hoja2" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$53</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="18">
   <si>
     <t>FOTO</t>
   </si>
@@ -34,6 +47,9 @@
   </si>
   <si>
     <t>Real</t>
+  </si>
+  <si>
+    <t>zarcillo</t>
   </si>
   <si>
     <t>pelicano juvenil</t>
@@ -51,32 +67,41 @@
     <t>cushuri adulto</t>
   </si>
   <si>
-    <t>Fecha tentativa salida</t>
+    <t>x_0.28</t>
   </si>
   <si>
-    <t>Nombres</t>
+    <t>a</t>
   </si>
   <si>
-    <t>Ximena Velez</t>
+    <t>Error</t>
   </si>
   <si>
-    <t>Vencimiento Emo</t>
+    <t>MAE</t>
   </si>
   <si>
-    <t>Vencimiento SCTR</t>
+    <t>abs(Error)</t>
   </si>
   <si>
-    <t>…</t>
+    <t>Error^2</t>
   </si>
   <si>
-    <t>zarcillo</t>
+    <t>RMSE</t>
+  </si>
+  <si>
+    <t>sMAPE</t>
+  </si>
+  <si>
+    <t>Smape</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,6 +111,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -110,18 +142,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -137,9 +171,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -177,9 +211,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -212,26 +246,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -264,26 +281,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -457,17 +457,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N53"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C53"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -478,606 +474,1711 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C2">
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C5">
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C6">
         <v>17</v>
       </c>
-      <c r="J6" t="s">
-        <v>8</v>
-      </c>
-      <c r="K6" t="s">
-        <v>9</v>
-      </c>
-      <c r="L6" t="s">
-        <v>11</v>
-      </c>
-      <c r="M6" t="s">
-        <v>12</v>
-      </c>
-      <c r="N6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C7">
         <v>5</v>
       </c>
-      <c r="J7" s="2">
-        <v>46257</v>
-      </c>
-      <c r="K7" t="s">
-        <v>10</v>
-      </c>
-      <c r="L7" s="2">
-        <v>46244</v>
-      </c>
-      <c r="M7" s="2">
-        <v>46242</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C8">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>109</v>
       </c>
       <c r="B9" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C9">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>109</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C10">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>110</v>
       </c>
       <c r="B11" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C11">
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>110</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C12">
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>113</v>
       </c>
       <c r="B13" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>113</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C14">
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>118</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C15">
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>119</v>
       </c>
       <c r="B16" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C16">
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>119</v>
       </c>
       <c r="B17" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C17">
         <v>106</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>124</v>
       </c>
       <c r="B18" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C18">
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>124</v>
       </c>
       <c r="B19" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C19">
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>127</v>
       </c>
       <c r="B20" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C20">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>127</v>
       </c>
       <c r="B21" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C21">
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>949</v>
       </c>
       <c r="B22" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C22">
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>949</v>
       </c>
       <c r="B23" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C23">
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>955</v>
       </c>
       <c r="B24" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C24">
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>957</v>
       </c>
       <c r="B25" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C25">
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>957</v>
       </c>
       <c r="B26" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C26">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>957</v>
       </c>
       <c r="B27" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C27">
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>960</v>
       </c>
       <c r="B28" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C28">
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>960</v>
       </c>
       <c r="B29" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C29">
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>960</v>
       </c>
       <c r="B30" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C30">
         <v>30</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>960</v>
       </c>
       <c r="B31" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C31">
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>960</v>
       </c>
       <c r="B32" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C32">
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>964</v>
       </c>
       <c r="B33" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C33">
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>964</v>
       </c>
       <c r="B34" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C34">
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>964</v>
       </c>
       <c r="B35" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C35">
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>964</v>
       </c>
       <c r="B36" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C36">
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>968</v>
       </c>
       <c r="B37" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C37">
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>968</v>
       </c>
       <c r="B38" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C38">
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>981</v>
       </c>
       <c r="B39" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C39">
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>981</v>
       </c>
       <c r="B40" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C40">
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>981</v>
       </c>
       <c r="B41" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C41">
         <v>28</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>981</v>
       </c>
       <c r="B42" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C42">
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>985</v>
       </c>
       <c r="B43" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C43">
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>985</v>
       </c>
       <c r="B44" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C44">
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>985</v>
       </c>
       <c r="B45" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C45">
         <v>31</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>988</v>
       </c>
       <c r="B46" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C46">
         <v>60</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>988</v>
       </c>
       <c r="B47" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C47">
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>992</v>
       </c>
       <c r="B48" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C48">
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>992</v>
       </c>
       <c r="B49" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C49">
         <v>42</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>992</v>
       </c>
       <c r="B50" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C50">
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>994</v>
       </c>
       <c r="B51" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C51">
         <v>39</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>996</v>
       </c>
       <c r="B52" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C52">
         <v>18</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>998</v>
       </c>
       <c r="B53" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C53">
         <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C53" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C77BD49-1E9A-4DE6-B03B-5A85FC83F886}">
+  <dimension ref="A1:P26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2">
+        <v>47</v>
+      </c>
+      <c r="J2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K2" t="s">
+        <v>9</v>
+      </c>
+      <c r="L2" t="s">
+        <v>2</v>
+      </c>
+      <c r="M2" t="s">
+        <v>11</v>
+      </c>
+      <c r="N2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>45</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>44</v>
+      </c>
+      <c r="L3">
+        <f>VLOOKUP(J3,$A$1:$C$24,3,0)</f>
+        <v>47</v>
+      </c>
+      <c r="M3">
+        <f>(L3-K3)</f>
+        <v>3</v>
+      </c>
+      <c r="N3">
+        <f>ABS(M3)</f>
+        <v>3</v>
+      </c>
+      <c r="O3">
+        <f>N3^2</f>
+        <v>9</v>
+      </c>
+      <c r="P3">
+        <f>2*N3/(L3+K3)</f>
+        <v>6.5934065934065936E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>17</v>
+      </c>
+      <c r="J4">
+        <v>109</v>
+      </c>
+      <c r="K4">
+        <v>3</v>
+      </c>
+      <c r="L4">
+        <f t="shared" ref="L4:L26" si="0">VLOOKUP(J4,$A$1:$C$24,3,0)</f>
+        <v>8</v>
+      </c>
+      <c r="M4">
+        <f t="shared" ref="M4:M26" si="1">(L4-K4)</f>
+        <v>5</v>
+      </c>
+      <c r="N4">
+        <f t="shared" ref="N4:N26" si="2">ABS(M4)</f>
+        <v>5</v>
+      </c>
+      <c r="O4">
+        <f t="shared" ref="O4:O26" si="3">N4^2</f>
+        <v>25</v>
+      </c>
+      <c r="P4">
+        <f t="shared" ref="P4:P26" si="4">2*N4/(L4+K4)</f>
+        <v>0.90909090909090906</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="J5">
+        <v>110</v>
+      </c>
+      <c r="K5">
+        <v>52</v>
+      </c>
+      <c r="L5">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+      <c r="M5">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="O5">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="P5">
+        <f t="shared" si="4"/>
+        <v>1.9047619047619049E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>109</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6">
+        <f>AVERAGE(N3:N26)</f>
+        <v>2.6086956521739131</v>
+      </c>
+      <c r="J6">
+        <v>113</v>
+      </c>
+      <c r="K6">
+        <v>31</v>
+      </c>
+      <c r="L6">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+      <c r="M6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="O6">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="P6">
+        <f t="shared" si="4"/>
+        <v>6.25E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>110</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7">
+        <v>53</v>
+      </c>
+      <c r="F7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7">
+        <f>SQRT(AVERAGE(O3:O26))</f>
+        <v>3.4135280741548732</v>
+      </c>
+      <c r="J7">
+        <v>118</v>
+      </c>
+      <c r="K7">
+        <v>29</v>
+      </c>
+      <c r="L7">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="M7">
+        <f t="shared" si="1"/>
+        <v>-1</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="O7">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="P7">
+        <f t="shared" si="4"/>
+        <v>3.5087719298245612E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>113</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8">
+        <v>33</v>
+      </c>
+      <c r="F8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="2">
+        <f>AVERAGE(P3:P26)</f>
+        <v>0.13364999848823661</v>
+      </c>
+      <c r="J8">
+        <v>119</v>
+      </c>
+      <c r="K8">
+        <v>104</v>
+      </c>
+      <c r="L8">
+        <f t="shared" si="0"/>
+        <v>106</v>
+      </c>
+      <c r="M8">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="N8">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="O8">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="P8">
+        <f t="shared" si="4"/>
+        <v>1.9047619047619049E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>118</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9">
+        <v>28</v>
+      </c>
+      <c r="J9">
+        <v>124</v>
+      </c>
+      <c r="K9">
+        <v>43</v>
+      </c>
+      <c r="L9">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="M9">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="N9">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="O9">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="P9">
+        <f t="shared" si="4"/>
+        <v>2.2988505747126436E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>119</v>
+      </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>106</v>
+      </c>
+      <c r="J10">
+        <v>127</v>
+      </c>
+      <c r="K10">
+        <v>12</v>
+      </c>
+      <c r="L10">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="M10">
+        <f t="shared" si="1"/>
+        <v>-3</v>
+      </c>
+      <c r="N10">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="O10">
+        <f t="shared" si="3"/>
+        <v>9</v>
+      </c>
+      <c r="P10">
+        <f t="shared" si="4"/>
+        <v>0.2857142857142857</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>124</v>
+      </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>44</v>
+      </c>
+      <c r="J11">
+        <v>3</v>
+      </c>
+      <c r="K11">
+        <v>45</v>
+      </c>
+      <c r="L11">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="M11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>127</v>
+      </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>9</v>
+      </c>
+      <c r="J12">
+        <v>5</v>
+      </c>
+      <c r="K12">
+        <v>16</v>
+      </c>
+      <c r="L12">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="M12">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="N12">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="O12">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="P12">
+        <f t="shared" si="4"/>
+        <v>6.0606060606060608E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>949</v>
+      </c>
+      <c r="B13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>9</v>
+      </c>
+      <c r="J13">
+        <v>8</v>
+      </c>
+      <c r="K13">
+        <v>8</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="M13">
+        <f t="shared" si="1"/>
+        <v>-2</v>
+      </c>
+      <c r="N13">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="O13">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="P13">
+        <f t="shared" si="4"/>
+        <v>0.2857142857142857</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>955</v>
+      </c>
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>59</v>
+      </c>
+      <c r="J14">
+        <v>949</v>
+      </c>
+      <c r="K14">
+        <v>6</v>
+      </c>
+      <c r="L14">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="M14">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="N14">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="O14">
+        <f t="shared" si="3"/>
+        <v>9</v>
+      </c>
+      <c r="P14">
+        <f t="shared" si="4"/>
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>957</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>49</v>
+      </c>
+      <c r="J15">
+        <v>955</v>
+      </c>
+      <c r="K15">
+        <v>66</v>
+      </c>
+      <c r="L15">
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+      <c r="M15">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
+      <c r="N15">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="O15">
+        <f t="shared" si="3"/>
+        <v>49</v>
+      </c>
+      <c r="P15">
+        <f t="shared" si="4"/>
+        <v>0.112</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>960</v>
+      </c>
+      <c r="B16" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16">
+        <v>30</v>
+      </c>
+      <c r="J16">
+        <v>957</v>
+      </c>
+      <c r="K16">
+        <v>59</v>
+      </c>
+      <c r="L16">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+      <c r="M16">
+        <f t="shared" si="1"/>
+        <v>-10</v>
+      </c>
+      <c r="N16">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="O16">
+        <f t="shared" si="3"/>
+        <v>100</v>
+      </c>
+      <c r="P16">
+        <f t="shared" si="4"/>
+        <v>0.18518518518518517</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>964</v>
+      </c>
+      <c r="B17" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>25</v>
+      </c>
+      <c r="J17">
+        <v>960</v>
+      </c>
+      <c r="K17">
+        <v>32</v>
+      </c>
+      <c r="L17">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="M17">
+        <f t="shared" si="1"/>
+        <v>-2</v>
+      </c>
+      <c r="N17">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="O17">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="P17">
+        <f t="shared" si="4"/>
+        <v>6.4516129032258063E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>981</v>
+      </c>
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18">
+        <v>28</v>
+      </c>
+      <c r="J18">
+        <v>964</v>
+      </c>
+      <c r="K18">
+        <v>27</v>
+      </c>
+      <c r="L18">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="M18">
+        <f t="shared" si="1"/>
+        <v>-2</v>
+      </c>
+      <c r="N18">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="O18">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="4"/>
+        <v>7.6923076923076927E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>985</v>
+      </c>
+      <c r="B19" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>988</v>
+      </c>
+      <c r="B20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20">
+        <v>60</v>
+      </c>
+      <c r="J20">
+        <v>981</v>
+      </c>
+      <c r="K20">
+        <v>30</v>
+      </c>
+      <c r="L20">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="M20">
+        <f t="shared" si="1"/>
+        <v>-2</v>
+      </c>
+      <c r="N20">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="O20">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="P20">
+        <f t="shared" si="4"/>
+        <v>6.8965517241379309E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>992</v>
+      </c>
+      <c r="B21" t="s">
+        <v>3</v>
+      </c>
+      <c r="C21">
+        <v>42</v>
+      </c>
+      <c r="J21">
+        <v>985</v>
+      </c>
+      <c r="K21">
+        <v>28</v>
+      </c>
+      <c r="L21">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+      <c r="M21">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="N21">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="O21">
+        <f t="shared" si="3"/>
+        <v>9</v>
+      </c>
+      <c r="P21">
+        <f t="shared" si="4"/>
+        <v>0.10169491525423729</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>994</v>
+      </c>
+      <c r="B22" t="s">
+        <v>3</v>
+      </c>
+      <c r="C22">
+        <v>39</v>
+      </c>
+      <c r="J22">
+        <v>988</v>
+      </c>
+      <c r="K22">
+        <v>62</v>
+      </c>
+      <c r="L22">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+      <c r="M22">
+        <f t="shared" si="1"/>
+        <v>-2</v>
+      </c>
+      <c r="N22">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="O22">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="P22">
+        <f t="shared" si="4"/>
+        <v>3.2786885245901641E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>996</v>
+      </c>
+      <c r="B23" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23">
+        <v>18</v>
+      </c>
+      <c r="J23">
+        <v>992</v>
+      </c>
+      <c r="K23">
+        <v>46</v>
+      </c>
+      <c r="L23">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="M23">
+        <f t="shared" si="1"/>
+        <v>-4</v>
+      </c>
+      <c r="N23">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="O23">
+        <f t="shared" si="3"/>
+        <v>16</v>
+      </c>
+      <c r="P23">
+        <f t="shared" si="4"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>998</v>
+      </c>
+      <c r="B24" t="s">
+        <v>3</v>
+      </c>
+      <c r="C24">
+        <v>10</v>
+      </c>
+      <c r="J24">
+        <v>994</v>
+      </c>
+      <c r="K24">
+        <v>36</v>
+      </c>
+      <c r="L24">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+      <c r="M24">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="N24">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="O24">
+        <f t="shared" si="3"/>
+        <v>9</v>
+      </c>
+      <c r="P24">
+        <f t="shared" si="4"/>
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="J25">
+        <v>996</v>
+      </c>
+      <c r="K25">
+        <v>18</v>
+      </c>
+      <c r="L25">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="M25">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="N25">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O25">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="P25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="J26">
+        <v>998</v>
+      </c>
+      <c r="K26">
+        <v>11</v>
+      </c>
+      <c r="L26">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="M26">
+        <f t="shared" si="1"/>
+        <v>-1</v>
+      </c>
+      <c r="N26">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="O26">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="P26">
+        <f t="shared" si="4"/>
+        <v>9.5238095238095233E-2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{564892C3-D231-4403-B960-28E7D0F05E2B}">
+  <dimension ref="A2:E26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>8</v>
+      </c>
+      <c r="E6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>109</v>
+      </c>
+      <c r="E7">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>110</v>
+      </c>
+      <c r="E8">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>113</v>
+      </c>
+      <c r="E9">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>118</v>
+      </c>
+      <c r="E10">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>119</v>
+      </c>
+      <c r="E11">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>124</v>
+      </c>
+      <c r="E12">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>127</v>
+      </c>
+      <c r="E13">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>949</v>
+      </c>
+      <c r="E14">
+        <v>949</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>955</v>
+      </c>
+      <c r="E15">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>957</v>
+      </c>
+      <c r="E16">
+        <v>957</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>960</v>
+      </c>
+      <c r="E17">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>964</v>
+      </c>
+      <c r="E18">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>981</v>
+      </c>
+      <c r="D19" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>985</v>
+      </c>
+      <c r="E20">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>988</v>
+      </c>
+      <c r="E21">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>992</v>
+      </c>
+      <c r="E22">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>994</v>
+      </c>
+      <c r="E23">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>996</v>
+      </c>
+      <c r="E24">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>998</v>
+      </c>
+      <c r="E25">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E26">
+        <v>998</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="E3:E26">
+    <sortCondition ref="E3:E26"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
ultimos cambios antes de la primera presentacion
</commit_message>
<xml_diff>
--- a/Estimacion_error/datos_aves_marinas/2025/abril/RLOF/conteos_reales.xlsx
+++ b/Estimacion_error/datos_aves_marinas/2025/abril/RLOF/conteos_reales.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renzo\Desktop\Estadística\Trabajos (laborales)\BMAP\Proyectos\conteo-aves-bmap\Estimacion_error\datos_aves_marinas\2025\abril\RLOF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renzo\Desktop\Data_Saiensss\Estadística\Trabajos (laborales)\BMAP\Proyectos\conteo-aves-bmap\Estimacion_error\datos_aves_marinas\2025\abril\RLOF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB89041-2E0D-4E98-B98E-A968A2768042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ADFACE2-5B62-4303-B912-96981E3E36A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,16 +29,17 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="19">
   <si>
     <t>FOTO</t>
   </si>
@@ -92,6 +93,9 @@
   </si>
   <si>
     <t>Smape</t>
+  </si>
+  <si>
+    <t>Preferir un modelo que subestime</t>
   </si>
 </sst>
 </file>
@@ -171,9 +175,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -211,9 +215,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -246,9 +250,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -281,9 +302,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -458,12 +496,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C53"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -474,7 +512,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -485,7 +523,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -496,7 +534,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -507,7 +545,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -518,7 +556,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -529,7 +567,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>8</v>
       </c>
@@ -540,7 +578,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>8</v>
       </c>
@@ -551,7 +589,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>109</v>
       </c>
@@ -562,7 +600,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>109</v>
       </c>
@@ -573,7 +611,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>110</v>
       </c>
@@ -584,7 +622,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>110</v>
       </c>
@@ -595,7 +633,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>113</v>
       </c>
@@ -606,7 +644,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>113</v>
       </c>
@@ -617,7 +655,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>118</v>
       </c>
@@ -628,7 +666,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>119</v>
       </c>
@@ -639,7 +677,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>119</v>
       </c>
@@ -650,7 +688,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>124</v>
       </c>
@@ -661,7 +699,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>124</v>
       </c>
@@ -672,7 +710,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>127</v>
       </c>
@@ -683,7 +721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>127</v>
       </c>
@@ -694,7 +732,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>949</v>
       </c>
@@ -705,7 +743,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>949</v>
       </c>
@@ -716,7 +754,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>955</v>
       </c>
@@ -727,7 +765,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>957</v>
       </c>
@@ -738,7 +776,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>957</v>
       </c>
@@ -749,7 +787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>957</v>
       </c>
@@ -760,7 +798,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>960</v>
       </c>
@@ -771,7 +809,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>960</v>
       </c>
@@ -782,7 +820,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>960</v>
       </c>
@@ -793,7 +831,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>960</v>
       </c>
@@ -804,7 +842,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>960</v>
       </c>
@@ -815,7 +853,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>964</v>
       </c>
@@ -826,7 +864,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>964</v>
       </c>
@@ -837,7 +875,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>964</v>
       </c>
@@ -848,7 +886,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>964</v>
       </c>
@@ -859,7 +897,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>968</v>
       </c>
@@ -870,7 +908,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>968</v>
       </c>
@@ -881,7 +919,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>981</v>
       </c>
@@ -892,7 +930,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>981</v>
       </c>
@@ -903,7 +941,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>981</v>
       </c>
@@ -914,7 +952,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>981</v>
       </c>
@@ -925,7 +963,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>985</v>
       </c>
@@ -936,7 +974,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>985</v>
       </c>
@@ -947,7 +985,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>985</v>
       </c>
@@ -958,7 +996,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>988</v>
       </c>
@@ -969,7 +1007,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>988</v>
       </c>
@@ -980,7 +1018,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>992</v>
       </c>
@@ -991,7 +1029,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>992</v>
       </c>
@@ -1002,7 +1040,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>992</v>
       </c>
@@ -1013,7 +1051,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>994</v>
       </c>
@@ -1024,7 +1062,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>996</v>
       </c>
@@ -1035,7 +1073,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>998</v>
       </c>
@@ -1055,9 +1093,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C77BD49-1E9A-4DE6-B03B-5A85FC83F886}">
   <dimension ref="A1:P26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1068,7 +1106,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1100,7 +1138,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>3</v>
       </c>
@@ -1137,7 +1175,7 @@
         <v>6.5934065934065936E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>5</v>
       </c>
@@ -1174,7 +1212,7 @@
         <v>0.90909090909090906</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>8</v>
       </c>
@@ -1211,7 +1249,7 @@
         <v>1.9047619047619049E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>109</v>
       </c>
@@ -1255,7 +1293,7 @@
         <v>6.25E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>110</v>
       </c>
@@ -1299,7 +1337,7 @@
         <v>3.5087719298245612E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>113</v>
       </c>
@@ -1343,7 +1381,7 @@
         <v>1.9047619047619049E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>118</v>
       </c>
@@ -1380,7 +1418,7 @@
         <v>2.2988505747126436E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>119</v>
       </c>
@@ -1417,7 +1455,7 @@
         <v>0.2857142857142857</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>124</v>
       </c>
@@ -1454,7 +1492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>127</v>
       </c>
@@ -1463,6 +1501,9 @@
       </c>
       <c r="C12">
         <v>9</v>
+      </c>
+      <c r="F12" t="s">
+        <v>18</v>
       </c>
       <c r="J12">
         <v>5</v>
@@ -1491,7 +1532,7 @@
         <v>6.0606060606060608E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>949</v>
       </c>
@@ -1528,7 +1569,7 @@
         <v>0.2857142857142857</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>955</v>
       </c>
@@ -1565,7 +1606,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>957</v>
       </c>
@@ -1602,7 +1643,7 @@
         <v>0.112</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>960</v>
       </c>
@@ -1611,6 +1652,12 @@
       </c>
       <c r="C16">
         <v>30</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>2</v>
       </c>
       <c r="J16">
         <v>957</v>
@@ -1639,7 +1686,7 @@
         <v>0.18518518518518517</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>964</v>
       </c>
@@ -1676,7 +1723,7 @@
         <v>6.4516129032258063E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>981</v>
       </c>
@@ -1713,7 +1760,7 @@
         <v>7.6923076923076927E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>985</v>
       </c>
@@ -1724,7 +1771,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>988</v>
       </c>
@@ -1761,7 +1808,7 @@
         <v>6.8965517241379309E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>992</v>
       </c>
@@ -1798,7 +1845,7 @@
         <v>0.10169491525423729</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>994</v>
       </c>
@@ -1835,7 +1882,7 @@
         <v>3.2786885245901641E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>996</v>
       </c>
@@ -1872,7 +1919,7 @@
         <v>9.0909090909090912E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>998</v>
       </c>
@@ -1909,7 +1956,7 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="J25">
         <v>996</v>
       </c>
@@ -1937,7 +1984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="J26">
         <v>998</v>
       </c>
@@ -1973,9 +2020,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{564892C3-D231-4403-B960-28E7D0F05E2B}">
   <dimension ref="A2:E26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1983,7 +2030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1991,7 +2038,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1999,7 +2046,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>5</v>
       </c>
@@ -2007,7 +2054,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>8</v>
       </c>
@@ -2015,7 +2062,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>109</v>
       </c>
@@ -2023,7 +2070,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>110</v>
       </c>
@@ -2031,7 +2078,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>113</v>
       </c>
@@ -2039,7 +2086,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>118</v>
       </c>
@@ -2047,7 +2094,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>119</v>
       </c>
@@ -2055,7 +2102,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>124</v>
       </c>
@@ -2063,7 +2110,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>127</v>
       </c>
@@ -2071,7 +2118,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>949</v>
       </c>
@@ -2079,7 +2126,7 @@
         <v>949</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>955</v>
       </c>
@@ -2087,7 +2134,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>957</v>
       </c>
@@ -2095,7 +2142,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>960</v>
       </c>
@@ -2103,7 +2150,7 @@
         <v>960</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>964</v>
       </c>
@@ -2111,7 +2158,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>981</v>
       </c>
@@ -2122,7 +2169,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>985</v>
       </c>
@@ -2130,7 +2177,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>988</v>
       </c>
@@ -2138,7 +2185,7 @@
         <v>985</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>992</v>
       </c>
@@ -2146,7 +2193,7 @@
         <v>988</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>994</v>
       </c>
@@ -2154,7 +2201,7 @@
         <v>992</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>996</v>
       </c>
@@ -2162,7 +2209,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>998</v>
       </c>
@@ -2170,7 +2217,7 @@
         <v>996</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E26">
         <v>998</v>
       </c>

</xml_diff>

<commit_message>
añadiendo estimaciones con sahi
</commit_message>
<xml_diff>
--- a/Estimacion_error/datos_aves_marinas/2025/abril/RLOF/conteos_reales.xlsx
+++ b/Estimacion_error/datos_aves_marinas/2025/abril/RLOF/conteos_reales.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renzo\Desktop\Data_Saiensss\Estadística\Trabajos (laborales)\BMAP\Proyectos\conteo-aves-bmap\Estimacion_error\datos_aves_marinas\2025\abril\RLOF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renzo\Desktop\Estadística\Trabajos (laborales)\BMAP\Proyectos\conteo-aves-bmap\Estimacion_error\datos_aves_marinas\2025\abril\RLOF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ADFACE2-5B62-4303-B912-96981E3E36A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C8BE49E-08FC-4C3D-90F7-CC8EB122DF5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Hoja2" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Hoja1!$J$32:$N$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$53</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -31,15 +32,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="22">
   <si>
     <t>FOTO</t>
   </si>
@@ -97,6 +95,15 @@
   <si>
     <t>Preferir un modelo que subestime</t>
   </si>
+  <si>
+    <t>sin sahi</t>
+  </si>
+  <si>
+    <t>Con sahi</t>
+  </si>
+  <si>
+    <t>x_0.46</t>
+  </si>
 </sst>
 </file>
 
@@ -150,12 +157,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -175,9 +184,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -215,9 +224,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -250,26 +259,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -302,26 +294,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -496,12 +471,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C53"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -512,7 +487,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -523,7 +498,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -534,7 +509,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -545,7 +520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -556,7 +531,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -567,7 +542,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>8</v>
       </c>
@@ -578,7 +553,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
@@ -589,7 +564,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>109</v>
       </c>
@@ -600,7 +575,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>109</v>
       </c>
@@ -611,7 +586,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>110</v>
       </c>
@@ -622,7 +597,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>110</v>
       </c>
@@ -633,7 +608,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>113</v>
       </c>
@@ -644,7 +619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>113</v>
       </c>
@@ -655,7 +630,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>118</v>
       </c>
@@ -666,7 +641,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>119</v>
       </c>
@@ -677,7 +652,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>119</v>
       </c>
@@ -688,7 +663,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>124</v>
       </c>
@@ -699,7 +674,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>124</v>
       </c>
@@ -710,7 +685,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>127</v>
       </c>
@@ -721,7 +696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>127</v>
       </c>
@@ -732,7 +707,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>949</v>
       </c>
@@ -743,7 +718,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>949</v>
       </c>
@@ -754,7 +729,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>955</v>
       </c>
@@ -765,7 +740,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>957</v>
       </c>
@@ -776,7 +751,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>957</v>
       </c>
@@ -787,7 +762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>957</v>
       </c>
@@ -798,7 +773,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>960</v>
       </c>
@@ -809,7 +784,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>960</v>
       </c>
@@ -820,7 +795,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>960</v>
       </c>
@@ -831,7 +806,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>960</v>
       </c>
@@ -842,7 +817,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>960</v>
       </c>
@@ -853,7 +828,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>964</v>
       </c>
@@ -864,7 +839,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>964</v>
       </c>
@@ -875,7 +850,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>964</v>
       </c>
@@ -886,7 +861,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>964</v>
       </c>
@@ -897,7 +872,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>968</v>
       </c>
@@ -908,7 +883,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>968</v>
       </c>
@@ -919,7 +894,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>981</v>
       </c>
@@ -930,7 +905,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>981</v>
       </c>
@@ -941,7 +916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>981</v>
       </c>
@@ -952,7 +927,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>981</v>
       </c>
@@ -963,7 +938,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>985</v>
       </c>
@@ -974,7 +949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>985</v>
       </c>
@@ -985,7 +960,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>985</v>
       </c>
@@ -996,7 +971,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>988</v>
       </c>
@@ -1007,7 +982,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>988</v>
       </c>
@@ -1018,7 +993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>992</v>
       </c>
@@ -1029,7 +1004,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>992</v>
       </c>
@@ -1040,7 +1015,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>992</v>
       </c>
@@ -1051,7 +1026,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>994</v>
       </c>
@@ -1062,7 +1037,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>996</v>
       </c>
@@ -1073,7 +1048,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>998</v>
       </c>
@@ -1092,10 +1067,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C77BD49-1E9A-4DE6-B03B-5A85FC83F886}">
-  <dimension ref="A1:P26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P56"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1105,8 +1080,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1138,7 +1116,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>3</v>
       </c>
@@ -1175,7 +1153,7 @@
         <v>6.5934065934065936E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>5</v>
       </c>
@@ -1212,7 +1190,7 @@
         <v>0.90909090909090906</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>8</v>
       </c>
@@ -1249,7 +1227,7 @@
         <v>1.9047619047619049E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>109</v>
       </c>
@@ -1293,7 +1271,7 @@
         <v>6.25E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>110</v>
       </c>
@@ -1337,7 +1315,7 @@
         <v>3.5087719298245612E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>113</v>
       </c>
@@ -1381,7 +1359,7 @@
         <v>1.9047619047619049E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>118</v>
       </c>
@@ -1418,7 +1396,7 @@
         <v>2.2988505747126436E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>119</v>
       </c>
@@ -1455,7 +1433,7 @@
         <v>0.2857142857142857</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>124</v>
       </c>
@@ -1492,7 +1470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>127</v>
       </c>
@@ -1501,9 +1479,6 @@
       </c>
       <c r="C12">
         <v>9</v>
-      </c>
-      <c r="F12" t="s">
-        <v>18</v>
       </c>
       <c r="J12">
         <v>5</v>
@@ -1532,7 +1507,7 @@
         <v>6.0606060606060608E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>949</v>
       </c>
@@ -1569,7 +1544,7 @@
         <v>0.2857142857142857</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>955</v>
       </c>
@@ -1606,7 +1581,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>957</v>
       </c>
@@ -1643,7 +1618,7 @@
         <v>0.112</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>960</v>
       </c>
@@ -1652,12 +1627,6 @@
       </c>
       <c r="C16">
         <v>30</v>
-      </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
-      <c r="G16">
-        <v>2</v>
       </c>
       <c r="J16">
         <v>957</v>
@@ -1686,7 +1655,7 @@
         <v>0.18518518518518517</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>964</v>
       </c>
@@ -1723,7 +1692,7 @@
         <v>6.4516129032258063E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>981</v>
       </c>
@@ -1760,7 +1729,7 @@
         <v>7.6923076923076927E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>985</v>
       </c>
@@ -1771,7 +1740,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>988</v>
       </c>
@@ -1808,7 +1777,7 @@
         <v>6.8965517241379309E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>992</v>
       </c>
@@ -1845,7 +1814,7 @@
         <v>0.10169491525423729</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>994</v>
       </c>
@@ -1882,7 +1851,7 @@
         <v>3.2786885245901641E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>996</v>
       </c>
@@ -1919,7 +1888,7 @@
         <v>9.0909090909090912E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>998</v>
       </c>
@@ -1956,7 +1925,7 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="J25">
         <v>996</v>
       </c>
@@ -1984,7 +1953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="J26">
         <v>998</v>
       </c>
@@ -2012,7 +1981,509 @@
         <v>9.5238095238095233E-2</v>
       </c>
     </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="J31" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="J32" t="s">
+        <v>0</v>
+      </c>
+      <c r="K32" t="s">
+        <v>21</v>
+      </c>
+      <c r="L32" t="s">
+        <v>2</v>
+      </c>
+      <c r="M32" t="s">
+        <v>13</v>
+      </c>
+      <c r="N32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="J33">
+        <v>1</v>
+      </c>
+      <c r="K33">
+        <v>49</v>
+      </c>
+      <c r="L33">
+        <f>VLOOKUP(J33,$A$1:$C$24,3,FALSE)</f>
+        <v>47</v>
+      </c>
+      <c r="M33">
+        <f>ABS(L33-K33)</f>
+        <v>2</v>
+      </c>
+      <c r="N33">
+        <f>2*(M33)/(K33+L33)</f>
+        <v>4.1666666666666664E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="F34" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" s="3">
+        <f>AVERAGE(M33:M56)</f>
+        <v>2.4782608695652173</v>
+      </c>
+      <c r="J34">
+        <v>109</v>
+      </c>
+      <c r="K34">
+        <v>8</v>
+      </c>
+      <c r="L34">
+        <f t="shared" ref="L34:L56" si="5">VLOOKUP(J34,$A$1:$C$24,3,FALSE)</f>
+        <v>8</v>
+      </c>
+      <c r="M34">
+        <f t="shared" ref="M34:M56" si="6">ABS(L34-K34)</f>
+        <v>0</v>
+      </c>
+      <c r="N34">
+        <f t="shared" ref="N34:N56" si="7">2*(M34)/(K34+L34)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="F35" t="s">
+        <v>17</v>
+      </c>
+      <c r="G35" s="4">
+        <f>AVERAGE(N33:N56)</f>
+        <v>6.8368799877003922E-2</v>
+      </c>
+      <c r="J35">
+        <v>110</v>
+      </c>
+      <c r="K35">
+        <v>51</v>
+      </c>
+      <c r="L35">
+        <f t="shared" si="5"/>
+        <v>53</v>
+      </c>
+      <c r="M35">
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="N35">
+        <f t="shared" si="7"/>
+        <v>3.8461538461538464E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="J36">
+        <v>113</v>
+      </c>
+      <c r="K36">
+        <v>31</v>
+      </c>
+      <c r="L36">
+        <f t="shared" si="5"/>
+        <v>33</v>
+      </c>
+      <c r="M36">
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="N36">
+        <f t="shared" si="7"/>
+        <v>6.25E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="J37">
+        <v>118</v>
+      </c>
+      <c r="K37">
+        <v>33</v>
+      </c>
+      <c r="L37">
+        <f t="shared" si="5"/>
+        <v>28</v>
+      </c>
+      <c r="M37">
+        <f t="shared" si="6"/>
+        <v>5</v>
+      </c>
+      <c r="N37">
+        <f t="shared" si="7"/>
+        <v>0.16393442622950818</v>
+      </c>
+    </row>
+    <row r="38" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="J38">
+        <v>119</v>
+      </c>
+      <c r="K38">
+        <v>101</v>
+      </c>
+      <c r="L38">
+        <f t="shared" si="5"/>
+        <v>106</v>
+      </c>
+      <c r="M38">
+        <f t="shared" si="6"/>
+        <v>5</v>
+      </c>
+      <c r="N38">
+        <f t="shared" si="7"/>
+        <v>4.8309178743961352E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="J39">
+        <v>124</v>
+      </c>
+      <c r="K39">
+        <v>45</v>
+      </c>
+      <c r="L39">
+        <f t="shared" si="5"/>
+        <v>44</v>
+      </c>
+      <c r="M39">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="N39">
+        <f t="shared" si="7"/>
+        <v>2.247191011235955E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="J40">
+        <v>127</v>
+      </c>
+      <c r="K40">
+        <v>11</v>
+      </c>
+      <c r="L40">
+        <f t="shared" si="5"/>
+        <v>9</v>
+      </c>
+      <c r="M40">
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="N40">
+        <f t="shared" si="7"/>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="41" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="J41">
+        <v>3</v>
+      </c>
+      <c r="K41">
+        <v>44</v>
+      </c>
+      <c r="L41">
+        <f t="shared" si="5"/>
+        <v>45</v>
+      </c>
+      <c r="M41">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="N41">
+        <f t="shared" si="7"/>
+        <v>2.247191011235955E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="J42">
+        <v>5</v>
+      </c>
+      <c r="K42">
+        <v>15</v>
+      </c>
+      <c r="L42">
+        <f t="shared" si="5"/>
+        <v>17</v>
+      </c>
+      <c r="M42">
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="N42">
+        <f t="shared" si="7"/>
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="43" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="J43">
+        <v>8</v>
+      </c>
+      <c r="K43">
+        <v>6</v>
+      </c>
+      <c r="L43">
+        <f t="shared" si="5"/>
+        <v>6</v>
+      </c>
+      <c r="M43">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N43">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="J44">
+        <v>949</v>
+      </c>
+      <c r="K44">
+        <v>10</v>
+      </c>
+      <c r="L44">
+        <f t="shared" si="5"/>
+        <v>9</v>
+      </c>
+      <c r="M44">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="N44">
+        <f t="shared" si="7"/>
+        <v>0.10526315789473684</v>
+      </c>
+    </row>
+    <row r="45" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="J45">
+        <v>955</v>
+      </c>
+      <c r="K45">
+        <v>53</v>
+      </c>
+      <c r="L45">
+        <f t="shared" si="5"/>
+        <v>59</v>
+      </c>
+      <c r="M45">
+        <f t="shared" si="6"/>
+        <v>6</v>
+      </c>
+      <c r="N45">
+        <f t="shared" si="7"/>
+        <v>0.10714285714285714</v>
+      </c>
+    </row>
+    <row r="46" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="J46">
+        <v>957</v>
+      </c>
+      <c r="K46">
+        <v>65</v>
+      </c>
+      <c r="L46">
+        <f t="shared" si="5"/>
+        <v>49</v>
+      </c>
+      <c r="M46">
+        <f t="shared" si="6"/>
+        <v>16</v>
+      </c>
+      <c r="N46">
+        <f t="shared" si="7"/>
+        <v>0.2807017543859649</v>
+      </c>
+    </row>
+    <row r="47" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="J47">
+        <v>960</v>
+      </c>
+      <c r="K47">
+        <v>32</v>
+      </c>
+      <c r="L47">
+        <f t="shared" si="5"/>
+        <v>30</v>
+      </c>
+      <c r="M47">
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="N47">
+        <f t="shared" si="7"/>
+        <v>6.4516129032258063E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="6:14" x14ac:dyDescent="0.3">
+      <c r="J48">
+        <v>964</v>
+      </c>
+      <c r="K48">
+        <v>26</v>
+      </c>
+      <c r="L48">
+        <f t="shared" si="5"/>
+        <v>25</v>
+      </c>
+      <c r="M48">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="N48">
+        <f t="shared" si="7"/>
+        <v>3.9215686274509803E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="10:14" x14ac:dyDescent="0.3">
+      <c r="J50">
+        <v>981</v>
+      </c>
+      <c r="K50">
+        <v>28</v>
+      </c>
+      <c r="L50">
+        <f t="shared" si="5"/>
+        <v>28</v>
+      </c>
+      <c r="M50">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N50">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="10:14" x14ac:dyDescent="0.3">
+      <c r="J51">
+        <v>985</v>
+      </c>
+      <c r="K51">
+        <v>31</v>
+      </c>
+      <c r="L51">
+        <f t="shared" si="5"/>
+        <v>31</v>
+      </c>
+      <c r="M51">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N51">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="10:14" x14ac:dyDescent="0.3">
+      <c r="J52">
+        <v>988</v>
+      </c>
+      <c r="K52">
+        <v>57</v>
+      </c>
+      <c r="L52">
+        <f t="shared" si="5"/>
+        <v>60</v>
+      </c>
+      <c r="M52">
+        <f t="shared" si="6"/>
+        <v>3</v>
+      </c>
+      <c r="N52">
+        <f t="shared" si="7"/>
+        <v>5.128205128205128E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="10:14" x14ac:dyDescent="0.3">
+      <c r="J53">
+        <v>992</v>
+      </c>
+      <c r="K53">
+        <v>45</v>
+      </c>
+      <c r="L53">
+        <f t="shared" si="5"/>
+        <v>42</v>
+      </c>
+      <c r="M53">
+        <f t="shared" si="6"/>
+        <v>3</v>
+      </c>
+      <c r="N53">
+        <f t="shared" si="7"/>
+        <v>6.8965517241379309E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="10:14" x14ac:dyDescent="0.3">
+      <c r="J54">
+        <v>994</v>
+      </c>
+      <c r="K54">
+        <v>40</v>
+      </c>
+      <c r="L54">
+        <f t="shared" si="5"/>
+        <v>39</v>
+      </c>
+      <c r="M54">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="N54">
+        <f t="shared" si="7"/>
+        <v>2.5316455696202531E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="10:14" x14ac:dyDescent="0.3">
+      <c r="J55">
+        <v>996</v>
+      </c>
+      <c r="K55">
+        <v>20</v>
+      </c>
+      <c r="L55">
+        <f t="shared" si="5"/>
+        <v>18</v>
+      </c>
+      <c r="M55">
+        <f t="shared" si="6"/>
+        <v>2</v>
+      </c>
+      <c r="N55">
+        <f t="shared" si="7"/>
+        <v>0.10526315789473684</v>
+      </c>
+    </row>
+    <row r="56" spans="10:14" x14ac:dyDescent="0.3">
+      <c r="J56">
+        <v>998</v>
+      </c>
+      <c r="K56">
+        <v>10</v>
+      </c>
+      <c r="L56">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="M56">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N56">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="J32:N48" xr:uid="{1C77BD49-1E9A-4DE6-B03B-5A85FC83F886}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2020,9 +2491,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{564892C3-D231-4403-B960-28E7D0F05E2B}">
   <dimension ref="A2:E26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2030,7 +2501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2038,7 +2509,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2046,7 +2517,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>5</v>
       </c>
@@ -2054,7 +2525,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>8</v>
       </c>
@@ -2062,7 +2533,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>109</v>
       </c>
@@ -2070,7 +2541,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>110</v>
       </c>
@@ -2078,7 +2549,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>113</v>
       </c>
@@ -2086,7 +2557,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>118</v>
       </c>
@@ -2094,7 +2565,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>119</v>
       </c>
@@ -2102,7 +2573,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>124</v>
       </c>
@@ -2110,7 +2581,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>127</v>
       </c>
@@ -2118,7 +2589,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>949</v>
       </c>
@@ -2126,7 +2597,7 @@
         <v>949</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>955</v>
       </c>
@@ -2134,7 +2605,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>957</v>
       </c>
@@ -2142,7 +2613,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>960</v>
       </c>
@@ -2150,7 +2621,7 @@
         <v>960</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>964</v>
       </c>
@@ -2158,7 +2629,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>981</v>
       </c>
@@ -2169,7 +2640,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>985</v>
       </c>
@@ -2177,7 +2648,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>988</v>
       </c>
@@ -2185,7 +2656,7 @@
         <v>985</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>992</v>
       </c>
@@ -2193,7 +2664,7 @@
         <v>988</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>994</v>
       </c>
@@ -2201,7 +2672,7 @@
         <v>992</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>996</v>
       </c>
@@ -2209,7 +2680,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>998</v>
       </c>
@@ -2217,7 +2688,7 @@
         <v>996</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E26">
         <v>998</v>
       </c>

</xml_diff>